<commit_message>
Apply emil-design-eng animation polish to Balance Cashout, extend scroll edge-fade to remaining tables
Balance: dropdown enter/exit transitions with transform-origin, active:scale press
feedback on all buttons, skeleton-to-data crossfade, KPI card stagger entrance, and
sort-header transition fixed to animate specific properties instead of `transition: all`.
Scroll edge-fade rolled out to Transfer Queue (Cashout + Send Money) and Send Money's
Balances/Opening/Settlement/Top Up tables, matching the pattern already used elsewhere.
Installs the emil-design-eng skill set and swaps in the new sidebar logo/favicon.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/SSP Line 2 Personal SendMoney Template .xlsx
+++ b/app/SSP Line 2 Personal SendMoney Template .xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ejboy\Downloads\Telegram Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ejboy\Desktop\dashbaord_project\app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD430842-9D33-4F33-80F6-75E8136E25F9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74E0D4C-80E0-44E9-B485-5ABAAB4EBA86}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="15465" windowHeight="7890" xr2:uid="{11DBCEFB-88F7-48A5-B32D-B2D8ED80C28F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{11DBCEFB-88F7-48A5-B32D-B2D8ED80C28F}"/>
   </bookViews>
   <sheets>
     <sheet name="Opening PS" sheetId="1" r:id="rId1"/>
@@ -637,7 +637,7 @@
     </row>
     <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H9" s="10">
-        <f>SUM(F:F)</f>
+        <f>SUM(C:C)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>